<commit_message>
Update reports with 10-9-PD data
Regenerated from the full daily export "10-9-PD.xls" (2,279 rows):
108 BK No outstanding, 310 containers across 8 depots (YJC DEPOT
back; ICD LKT and Sintanachote files removed as they have no data
in this list). No rows flagged for missing Pickup Name.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - UNITHAI CONTAINER TERMINAL.xlsx
+++ b/output/bkg pending - UNITHAI CONTAINER TERMINAL.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$V$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$V$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -613,7 +613,7 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260700892</t>
+          <t>HASLS22260901754</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610110500</t>
+          <t>202610111300</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
@@ -669,7 +669,8 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>STUFFING CARGO @UNITHAI DD.09/10/26 *CLS TIME CFS DD.09/10/26 - 17:00HRS.*</t>
+          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.09/10/26 CLS TIME CFS DD.09/10/26 - 17:00HRS.
+ </t>
         </is>
       </c>
       <c r="N2" s="2" t="n">
@@ -703,7 +704,7 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900303</t>
+          <t>HASLS22260902782</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -718,7 +719,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610110500</t>
+          <t>202610111300</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -729,7 +730,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -744,12 +745,12 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>CHOTIWAT MANUFACTURING PUBLIC COMPANY LIMITED</t>
+          <t>NEO AGRO BUSINESS CO.,LTD.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PET FOOD</t>
+          <t>MEDICAL EQUIPMENT</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -793,22 +794,22 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901654</t>
+          <t>HASLS22261000118</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SWAL</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>0152N</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610191500</t>
+          <t>202610111300</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -824,22 +825,22 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261009</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>MINERAL RESOURCES DEVELOPMENT CO., LTD.</t>
+          <t>SIAM MACHINERY AND EQUIPMENT CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>KAOLIN</t>
+          <t>DUCTILE CAST IRON ROLLS</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -849,12 +850,11 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.15/10/26 CLS TIME CFS DD.16/10/26 - 17:00HRS.
-</t>
+          <t>STUFFING @UNITHAI DD.09/10/26 *CLS TIME CFS DD.09/10/26 - 17:00HRS.*</t>
         </is>
       </c>
       <c r="N4" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>0</v>
@@ -884,7 +884,7 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901754</t>
+          <t>HASLS22261000141</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610110500</t>
+          <t>202610111300</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -910,12 +910,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -925,33 +925,32 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>SIAM BROTHERS CORP.,LTD.</t>
+          <t>UNICORD PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>FISHING NETS</t>
+          <t>CANNED GOOD</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>REQ: GOOD &amp; CLEAN CONTAINER,NO LEAK,NO RUST,NO SMELL,NO BURR,NOT WET,GOOD FLOOR.</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.09/10/26 CLS TIME CFS DD.09/10/26 - 17:00HRS.
- </t>
+          <t>STUFFING @UNITHAI DD.09/10/26 *CLS TIME CFS DD.09/10/26 - 17:00HRS.*</t>
         </is>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O5" s="2" t="n">
         <v>0</v>
       </c>
       <c r="P5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="2" t="n">
         <v>0</v>
@@ -975,22 +974,22 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901757</t>
+          <t>HASLS22261000609</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SWAL</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2616N</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610191500</t>
+          <t>202610150400</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1006,43 +1005,43 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20261016</t>
+          <t>20261009</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>SIAM BROTHERS CORP.,LTD.</t>
+          <t>SADESA (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>FISHING NETS</t>
+          <t>COW LEATHER</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>REQ: GOOD &amp; CLEAN CONTAINER,NO LEAK,NO RUST,NO SMELL,NO BURR,NOT WET,GOOD FLOOR.</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.16/10/26 CLS TIME CFS DD.16/10/26 - 17:00HRS.
+          <t xml:space="preserve">STUFFING @ UNITHAI DD 09/10/26 CLS TIME 12/10 @17.00HRS 
 </t>
         </is>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>0</v>
@@ -1064,740 +1063,105 @@
       </c>
     </row>
     <row r="7" ht="13" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260901991</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>SWAL</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>202610191500</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>20261016</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>CHINCHANA INDUSTRIES (THAILAND) CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>BARIUM SULPHATE WHITE ROCK 20A NON DG HS-CODE.251110.00</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>6
-RQE:CLEAN AND DRY UPGRADE CONT*</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STUFFING CARGO @UINTHAI DD.16/10/26 CLS TIME CFS DD.16/10/26 - 17:00HRS.
-</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" ht="13" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902782</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>DJCF</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>0152N</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>202610110500</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>NEO AGRO BUSINESS CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>MEDICAL EQUIPMENT</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>STUFFING @UNITHAI DD.09/10/26 *CLS TIME CFS DD.09/10/26 - 17:00HRS.*</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902785</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>KUS</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>2616N</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>202610141100</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>ISTO IMPORT &amp; EXPORT CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>THAI FODDSTUFF</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.09/10/26 CLS TIME CFS DD.12/10/26 - 17:00HRS.
-</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="2" t="n">
-        <v>0</v>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
+      <c r="K7" s="3" t="n"/>
+      <c r="L7" s="3" t="n"/>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3">
+        <f>SUM(N2:N6)</f>
+        <v/>
+      </c>
+      <c r="O7" s="3">
+        <f>SUM(O2:O6)</f>
+        <v/>
+      </c>
+      <c r="P7" s="3">
+        <f>SUM(P2:P6)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="3">
+        <f>SUM(Q2:Q6)</f>
+        <v/>
+      </c>
+      <c r="R7" s="3">
+        <f>SUM(R2:R6)</f>
+        <v/>
+      </c>
+      <c r="S7" s="3">
+        <f>SUM(S2:S6)</f>
+        <v/>
+      </c>
+      <c r="T7" s="3">
+        <f>SUM(T2:T6)</f>
+        <v/>
+      </c>
+      <c r="U7" s="3">
+        <f>SUM(U2:U6)</f>
+        <v/>
+      </c>
+      <c r="V7" s="3">
+        <f>SUM(V2:V6)</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="13" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22260902820</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>SWAL</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>202610191500</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>20261015</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>CHAI SAN SAN TRADING LIMITED</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>NOODLE</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.15/10/26 CLS TIME CFS DD.16/10/26 - 17:00HRS.
-</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V10" s="2" t="n">
-        <v>0</v>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902822</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>PGPO</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>202610150800</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>20261013</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>CHAI SAN SAN TRADING LIMITED</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>NOODLE</t>
-        </is>
-      </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">STUFFING CARGO @UNITHAI DD.12/10/26 CLS TIME CFS DD.12/10/26 - 17:00HRS.
-</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" s="2" t="n">
-        <v>0</v>
+          <t>UNITHAI CONTAINER TERMINAL</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261000118</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>DJCF</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>0152N</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>202610110500</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>SIAM MACHINERY AND EQUIPMENT CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>DUCTILE CAST IRON ROLLS</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>STUFFING @UNITHAI DD.09/10/26 *CLS TIME CFS DD.09/10/26 - 17:00HRS.*</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261000141</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>DJCF</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>0152N</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>202610110500</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>KRINC</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>UNICORD PUBLIC COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>CANNED GOOD</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>STUFFING @UNITHAI DD.09/10/26 *CLS TIME CFS DD.09/10/26 - 17:00HRS.*</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="3">
-        <f>SUM(N2:N13)</f>
-        <v/>
-      </c>
-      <c r="O14" s="3">
-        <f>SUM(O2:O13)</f>
-        <v/>
-      </c>
-      <c r="P14" s="3">
-        <f>SUM(P2:P13)</f>
-        <v/>
-      </c>
-      <c r="Q14" s="3">
-        <f>SUM(Q2:Q13)</f>
-        <v/>
-      </c>
-      <c r="R14" s="3">
-        <f>SUM(R2:R13)</f>
-        <v/>
-      </c>
-      <c r="S14" s="3">
-        <f>SUM(S2:S13)</f>
-        <v/>
-      </c>
-      <c r="T14" s="3">
-        <f>SUM(T2:T13)</f>
-        <v/>
-      </c>
-      <c r="U14" s="3">
-        <f>SUM(U2:U13)</f>
-        <v/>
-      </c>
-      <c r="V14" s="3">
-        <f>SUM(V2:V13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="13" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="13" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>UNITHAI CONTAINER TERMINAL</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" ht="13" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>15</v>
+      <c r="B12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V13"/>
+  <autoFilter ref="A1:V6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>